<commit_message>
verified and tested matcher algorithm! :)
</commit_message>
<xml_diff>
--- a/results/rounds.xlsx
+++ b/results/rounds.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1127,678 +1127,6 @@
         <v>56.94</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>3</v>
-      </c>
-      <c r="B34" t="n">
-        <v>1</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Helen Yoon_20260116_172314</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>51.33</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>3</v>
-      </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Tiffany Zhong_20260117_003118</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>51.78</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>3</v>
-      </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Jonathan C_20260116_171814</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>42.17</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>3</v>
-      </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Ben DeGioia_20260116_172416</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>43.86</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>3</v>
-      </c>
-      <c r="B38" t="n">
-        <v>2</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Grace Lee_20260117_114907</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>52.05</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>3</v>
-      </c>
-      <c r="B39" t="n">
-        <v>2</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Vianca Yoon_20260116_193608</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>53.2</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>3</v>
-      </c>
-      <c r="B40" t="n">
-        <v>2</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Nora_20260117_082206</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>48.58</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>3</v>
-      </c>
-      <c r="B41" t="n">
-        <v>2</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Haydn_20260117_104416</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>49.56</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>3</v>
-      </c>
-      <c r="B42" t="n">
-        <v>3</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Chinenye Victoria Onukaogu_20260116_171323</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>44.22</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>3</v>
-      </c>
-      <c r="B43" t="n">
-        <v>3</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>KP Ko_20260116_214646</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>47.78</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>3</v>
-      </c>
-      <c r="B44" t="n">
-        <v>3</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>James Ahn_20260116_163855</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>53.38</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>3</v>
-      </c>
-      <c r="B45" t="n">
-        <v>3</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Jeremy Vinarao_20260117_055638</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>3</v>
-      </c>
-      <c r="B46" t="n">
-        <v>4</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Catherine Meng_20260116_165524</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E46" t="n">
-        <v>49.47</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>3</v>
-      </c>
-      <c r="B47" t="n">
-        <v>4</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Joanna Park_20260117_103454</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>50.53</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>3</v>
-      </c>
-      <c r="B48" t="n">
-        <v>4</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Daniel Choi_20260116_184114</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>55.34</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>3</v>
-      </c>
-      <c r="B49" t="n">
-        <v>4</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Zoe Liao_20260116_231803</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>56.94</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>4</v>
-      </c>
-      <c r="B50" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Grace Lee_20260117_114907</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>52.05</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>4</v>
-      </c>
-      <c r="B51" t="n">
-        <v>1</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Vianca Yoon_20260116_193608</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E51" t="n">
-        <v>53.2</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>4</v>
-      </c>
-      <c r="B52" t="n">
-        <v>1</v>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Jonathan C_20260116_171814</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E52" t="n">
-        <v>42.17</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>4</v>
-      </c>
-      <c r="B53" t="n">
-        <v>1</v>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Ben DeGioia_20260116_172416</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E53" t="n">
-        <v>43.86</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>4</v>
-      </c>
-      <c r="B54" t="n">
-        <v>2</v>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Chinenye Victoria Onukaogu_20260116_171323</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E54" t="n">
-        <v>44.22</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>4</v>
-      </c>
-      <c r="B55" t="n">
-        <v>2</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>KP Ko_20260116_214646</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E55" t="n">
-        <v>47.78</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>4</v>
-      </c>
-      <c r="B56" t="n">
-        <v>2</v>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Nora_20260117_082206</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E56" t="n">
-        <v>48.58</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>4</v>
-      </c>
-      <c r="B57" t="n">
-        <v>2</v>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Haydn_20260117_104416</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E57" t="n">
-        <v>49.56</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>4</v>
-      </c>
-      <c r="B58" t="n">
-        <v>3</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Catherine Meng_20260116_165524</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E58" t="n">
-        <v>49.47</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>4</v>
-      </c>
-      <c r="B59" t="n">
-        <v>3</v>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Joanna Park_20260117_103454</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E59" t="n">
-        <v>50.53</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>4</v>
-      </c>
-      <c r="B60" t="n">
-        <v>3</v>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>James Ahn_20260116_163855</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E60" t="n">
-        <v>53.38</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B61" t="n">
-        <v>3</v>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Jeremy Vinarao_20260117_055638</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n">
-        <v>4</v>
-      </c>
-      <c r="B62" t="n">
-        <v>4</v>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Helen Yoon_20260116_172314</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E62" t="n">
-        <v>51.33</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="n">
-        <v>4</v>
-      </c>
-      <c r="B63" t="n">
-        <v>4</v>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Tiffany Zhong_20260117_003118</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E63" t="n">
-        <v>51.78</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="n">
-        <v>4</v>
-      </c>
-      <c r="B64" t="n">
-        <v>4</v>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Daniel Choi_20260116_184114</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E64" t="n">
-        <v>55.34</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="n">
-        <v>4</v>
-      </c>
-      <c r="B65" t="n">
-        <v>4</v>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Zoe Liao_20260116_231803</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E65" t="n">
-        <v>56.94</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>